<commit_message>
Du lieu quet 09/10 (dashboard)
</commit_message>
<xml_diff>
--- a/data/bao_cao_dau_tu_20261009.xlsx
+++ b/data/bao_cao_dau_tu_20261009.xlsx
@@ -649,27 +649,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1.53%</t>
+          <t>1.45%</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+62.6%</t>
+          <t>+64.4%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>+34.2%</t>
+          <t>+36.3%</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>+12.1%</t>
+          <t>+7.5%</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>+6.6%</t>
+          <t>+6.3%</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -711,31 +711,31 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>31450</v>
+        <v>31150</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1.91%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>+4.9%</t>
+          <t>+6.7%</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>+11.2%</t>
+          <t>+9.2%</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>+2.8%</t>
+          <t>+1.9%</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -777,31 +777,31 @@
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>32000</v>
+        <v>31050</v>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>4.12%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>+57.4%</t>
+          <t>+58.8%</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>+25.0%</t>
+          <t>+23.4%</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>+35.1%</t>
+          <t>+24.9%</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>+21.8%</t>
+          <t>+19.7%</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -843,31 +843,31 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>47750</v>
+        <v>47250</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>3.92%</t>
+          <t>3.80%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>-5.6%</t>
+          <t>+3.4%</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+12.8%</t>
+          <t>+9.4%</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>+29.9%</t>
+          <t>+30.1%</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>+21.5%</t>
+          <t>+13.1%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -909,11 +909,11 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>39200</v>
+        <v>36500</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2.68%</t>
+          <t>3.07%</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -923,17 +923,17 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+29.2%</t>
+          <t>+20.9%</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>+27.6%</t>
+          <t>+19.4%</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>+15.7%</t>
+          <t>+7.5%</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>16700</v>
+        <v>16900</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>5.08%</t>
+          <t>5.15%</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+19.0%</t>
+          <t>+18.9%</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>+40.8%</t>
+          <t>+40.7%</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>+37.0%</t>
+          <t>+40.0%</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>+25.1%</t>
+          <t>+28.5%</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1041,11 +1041,11 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>150900</v>
+        <v>149600</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>3.72%</t>
+          <t>3.73%</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1055,17 +1055,17 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>+2.3%</t>
+          <t>+3.8%</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>+35.8%</t>
+          <t>+35.3%</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>+12.2%</t>
+          <t>+12.0%</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1107,31 +1107,31 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>54200</v>
+        <v>55000</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>2.27%</t>
+          <t>2.38%</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+7.3%</t>
+          <t>+6.3%</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>+12.7%</t>
+          <t>+15.2%</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>+11.2%</t>
+          <t>+14.1%</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>+12.3%</t>
+          <t>+14.8%</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1173,31 +1173,31 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>23600</v>
+        <v>23150</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>3.20%</t>
+          <t>3.17%</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
+          <t>+7.9%</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
           <t>+6.9%</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>+9.2%</t>
-        </is>
-      </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>+3.2%</t>
+          <t>+1.3%</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>-5.6%</t>
+          <t>-6.8%</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1239,31 +1239,31 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>28000</v>
+        <v>22400</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2.15%</t>
+          <t>2.54%</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+6.7%</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+7.9%</t>
+          <t>+11.7%</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>+7.8%</t>
+          <t>+12.4%</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>+6.6%</t>
+          <t>+11.2%</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1305,31 +1305,31 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>17600</v>
+        <v>17650</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2.46%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+81.3%</t>
+          <t>+76.6%</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+48.7%</t>
+          <t>+51.6%</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>+28.7%</t>
+          <t>+31.5%</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>+7.2%</t>
+          <t>+8.4%</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1371,31 +1371,31 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>40650</v>
+        <v>40700</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>3.93%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>-11.8%</t>
+          <t>-14.1%</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>-14.0%</t>
+          <t>-8.1%</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-17.3%</t>
+          <t>-16.6%</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-10.8%</t>
+          <t>-10.3%</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1437,31 +1437,31 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>14750</v>
+        <v>14600</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2.89%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+5.9%</t>
+          <t>+7.5%</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+49.6%</t>
+          <t>+44.8%</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>+16.8%</t>
+          <t>+15.2%</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>+19.2%</t>
+          <t>+17.9%</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1503,31 +1503,31 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>68200</v>
+        <v>67900</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>6.17%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
+          <t>+98.5%</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+48.1%</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
           <t>+93.7%</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>+48.1%</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>+98.1%</t>
-        </is>
-      </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>+49.3%</t>
+          <t>+50.8%</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1569,31 +1569,31 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>47950</v>
+        <v>48000</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+39.7%</t>
+          <t>+38.0%</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>-3.6%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>+4.8%</t>
+          <t>+4.4%</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>+4.1%</t>
+          <t>+5.1%</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1635,31 +1635,31 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>16600</v>
+        <v>17100</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>6.89%</t>
+          <t>7.12%</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>-29.7%</t>
+          <t>-28.5%</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+51.5%</t>
+          <t>+56.7%</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>+16.9%</t>
+          <t>+23.7%</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>+45.5%</t>
+          <t>+48.9%</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1701,31 +1701,31 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>49400</v>
+        <v>50500</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>6.59%</t>
+          <t>6.61%</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+72.9%</t>
+          <t>+73.4%</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+50.9%</t>
+          <t>+49.0%</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>+40.8%</t>
+          <t>+39.7%</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>+35.0%</t>
+          <t>+36.1%</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1767,31 +1767,31 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>49900</v>
+        <v>49100</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>3.95%</t>
+          <t>4.07%</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>+26.1%</t>
+          <t>+24.5%</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+52.0%</t>
+          <t>+51.2%</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>+37.2%</t>
+          <t>+34.6%</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>+13.8%</t>
+          <t>+12.8%</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1833,31 +1833,31 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>25000</v>
+        <v>24100</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>5.44%</t>
+          <t>5.63%</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+24.9%</t>
+          <t>+25.0%</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+80.0%</t>
+          <t>+72.9%</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>+60.3%</t>
+          <t>+53.4%</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>+43.5%</t>
+          <t>+38.1%</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1899,31 +1899,31 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>25550</v>
+        <v>25200</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>4.72%</t>
+          <t>4.67%</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>+17.8%</t>
+          <t>+23.6%</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>+30.8%</t>
+          <t>+27.2%</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>+37.5%</t>
+          <t>+35.3%</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>+26.5%</t>
+          <t>+21.0%</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1965,31 +1965,31 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>52200</v>
+        <v>51800</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>1.78%</t>
+          <t>1.89%</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>+2.3%</t>
+          <t>+1.5%</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>+13.8%</t>
+          <t>+17.3%</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>+14.8%</t>
+          <t>+14.0%</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>+11.1%</t>
+          <t>+10.9%</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -2031,31 +2031,31 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>22800</v>
+        <v>22850</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>1.60%</t>
+          <t>1.56%</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>-9.0%</t>
+          <t>-9.3%</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+7.0%</t>
+          <t>+11.6%</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>+13.5%</t>
+          <t>+13.3%</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>+4.0%</t>
+          <t>+4.3%</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -2097,31 +2097,31 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>17100</v>
+        <v>16800</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>5.73%</t>
+          <t>5.44%</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>-0.0%</t>
+          <t>+3.0%</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>+19.0%</t>
+          <t>+20.3%</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>+10.5%</t>
+          <t>+11.1%</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>+1.4%</t>
+          <t>-1.5%</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -2167,27 +2167,27 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>2.81%</t>
+          <t>2.82%</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+20.1%</t>
+          <t>+25.7%</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>+5.4%</t>
+          <t>+3.2%</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>+1.1%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>-7.4%</t>
+          <t>-8.6%</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2229,31 +2229,31 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>54800</v>
+        <v>54000</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>2.66%</t>
+          <t>2.62%</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>+1.3%</t>
+          <t>+0.9%</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+12.2%</t>
+          <t>+10.6%</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>+20.1%</t>
+          <t>+18.9%</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>+13.6%</t>
+          <t>+13.5%</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -2299,27 +2299,27 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>1.21%</t>
+          <t>1.19%</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>-6.3%</t>
+          <t>-7.7%</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+9.6%</t>
+          <t>+13.1%</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>+13.3%</t>
+          <t>+12.9%</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>+8.1%</t>
+          <t>+9.0%</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -2361,31 +2361,31 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>65700</v>
+        <v>66000</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>3.55%</t>
+          <t>3.33%</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>+41.3%</t>
+          <t>+40.7%</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+15.0%</t>
+          <t>+12.7%</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>-6.2%</t>
+          <t>-5.5%</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>-4.1%</t>
+          <t>-4.6%</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -2427,31 +2427,31 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>228000</v>
+        <v>225500</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>3.26%</t>
+          <t>3.05%</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>+179.2%</t>
+          <t>+169.5%</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+55.3%</t>
+          <t>+48.2%</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>+9.5%</t>
+          <t>+7.8%</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>-3.1%</t>
+          <t>-3.8%</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -2493,16 +2493,16 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>23450</v>
+        <v>23800</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2.60%</t>
+          <t>2.55%</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>-18.0%</t>
+          <t>-16.3%</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2512,12 +2512,12 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>+12.7%</t>
+          <t>+15.8%</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>+12.7%</t>
+          <t>+14.2%</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2559,31 +2559,31 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>56600</v>
+        <v>55500</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>3.23%</t>
+          <t>3.07%</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>+4.3%</t>
+          <t>+8.8%</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+4.4%</t>
+          <t>+6.5%</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>+7.4%</t>
+          <t>+2.6%</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>-4.5%</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2625,31 +2625,31 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>20200</v>
+        <v>20300</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>1.13%</t>
+          <t>1.06%</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>+0.9%</t>
+          <t>+0.3%</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>-3.2%</t>
+          <t>+1.2%</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>+5.2%</t>
+          <t>+4.8%</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>+3.4%</t>
+          <t>+4.7%</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -2691,21 +2691,21 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>83000</v>
+        <v>82000</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>4.38%</t>
+          <t>4.41%</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>+293.7%</t>
+          <t>+290.8%</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>+34.2%</t>
+          <t>+40.9%</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>-1.6%</t>
+          <t>-2.4%</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>14750</v>
+        <v>14600</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13333</v>
@@ -2828,7 +2828,7 @@
         <v>140</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>2065000</v>
+        <v>2044000</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -3312,7 +3312,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HDB</t>
+          <t>GMD</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -3332,16 +3332,20 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>chua</t>
+          <t>dat</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>chua</t>
+          <t>cho</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
           <t>N</t>
@@ -3366,7 +3370,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GMD</t>
+          <t>HHP</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -3386,20 +3390,16 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>dat</t>
+          <t>chua</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>cho</t>
+          <t>chua</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr">
         <is>
           <t>N</t>
@@ -3424,7 +3424,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HHP</t>
+          <t>HDB</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -3584,124 +3584,124 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>DHC</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>STB</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>loai</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>ro co ban chua chot</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>loai</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>cho</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>PHU QUYET BUOC 3 — phieu tham dinh 13/09/2026, het han 12/12/2026. Nam cong phu quyet DEU KHONG bat; phieu chet o DIEM: truc A 0 + truc B 1 + truc C 0 = 1/6, vua duoi tran 2 vua co truc bang 0 (thoa ca hai dieu kien phu quyet). TRUC A = 0: ROE 2025 10,34% va TTM den 30/06/2026 ~5,2% deu duoi COE 15,38% — hai trong ba ky do gan nhat duoi chi phi von. Nam duy nhat vuot la 2024 (20,03%) va no vuot nho chi phi tin dung 0,39% tren du no binh quan (so 1,95% cua 2025), dung nam ma NHNN ket luan trich lap du phong chua dung quy dinh — diem quan sat duy nhat chong lai muc 0 lai la diem quan sat da bi co quan quan ly dat dau hoi. TRUC C = 0: QD 1869 (cong bo 16-17/08/2025, phat 975 trieu, 6 vi pham, 28 kien nghi) ket luan PHAN LOAI TAI SAN CO va TRICH LAP DU PHONG chua dung quy dinh — ben co toan bo ho so tin dung noi rang so lieu dau vao sai, la dang bang chung nguoc nang nhat co the co cho mot truc cham chat luong cong bo. Cong them 3.789 ty 'dich vu khac' (21,7% tong thu nhap hoat dong 6T/2026, +2.408 ty YoY) khong co thuyet minh. TRUC B = 1: nen tien gui ban le 647.939 ty voi LDR 98,2% la loi the cau truc that, nhung CHUA quy doi duoc thanh bien co loi — CASA 18,9% (2022) -&gt; 16,5%, chi phi von tren tai san sinh loi 3,81% (2024) -&gt; 4,42%, NIM 2,81% da THAP HON binh quan nganh 2,87%, nhan su 18.659 -&gt; 13.078. Thay doi cau truc nganh bat loi nhung do duoc nen khong roi xuong 0. DO BEN KET LUAN: doc rong tay nhat cho truc A (chi lay 3 nam tai chinh 2023-2025, vut bo ky soat xet moi nhat) van ra 2/6 = VAN PHU QUYET. Phai dong thoi bo qua ky soat xet moi nhat VA ket luan thanh tra VA cham truc B muc 2 (du CASA/NIM deu di xuong) moi ra duoc 'Dat'.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Bán</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Khac</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>dat</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>ro co ban chua chot</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>dat</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>dat</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>BA LUAN DIEM — phieu 13/09/2026, nhip C. Chi viet duoc vi nhip B DAT; day la ma DUY NHAT trong bon phieu di het quy trinh. (1) CU SOC PHONG KHE LA CU SOC CUNG VA DA CHUYEN THANH BIEN LOI NHUAN, khong dung o tin tuc: ~200 co so dong cua tu dau 2025 rut ~2 trieu tan/nam = 22-26% nang luc nganh, thieu hut 601.000 tan trong 7 thang dau 2026. Gia ban giay cua DHC di tu ~9.002 d/kg (Q2/2025) len 10.442 d/kg (Q2/2026), +16%. Co che: DHC song bang CHENH LECH gia, gia OCC ton kho dung o 4.800 d/kg trong khi gia ban tang 1.440 d/kg, nen gan nhu toan bo muc tang roi thang xuong bien — bien gop 11,8% (2024) -&gt; 24,2% (6T/2026). Noi vao dinh gia: bien gop 23,5% cua 2026F la GIA DINH TRUNG TAM cua toan bo mo hinh. (2) DHC CHUYEN LOI NHUAN THANH TIEN TOT HON MOI MA TRONG NHOM SO SANH, VA DIEU DO DA DUOC KIEM O DAY CHU KY CHU KHONG PHAI O DINH: dong tien HD cong don 2023-2025 = 144,2% LNST cong don; nam te nhat 2024 khi bien gop roi xuong 11,8% dong tien van 656,2 ty = 2,7 lan LNST 242,2 ty; no rong AM 339 ty tai 30/06/2026. Co che: vong quay ngan vi mua va ban deu giao ngay, khau hao 111,1 ty/nam chay tren day chuyen DA TRA XONG, va khong mot dong phai thu ben lien quan nao phai cho thu. Noi vao dinh gia: day la thu cho phep tai tro 1.814 ty con lai cua Giao Long 3 MA KHONG CAN TANG VON — tuc khong pha loang nguoi dang cam co phieu. (3) UU DAI THUE HET HAN LA BUOC NHAY CHI PHI VINH VIEN phai neo vao MOI nam du phong, khong phai bien dong mot lan: uu dai giam 50% cua Giao Long giai doan 2 het hieu luc 31/12/2025; thue suat hieu dung di tu 14,0% (2025) len 19,5% (6T/2026), chi phi thue hien hanh +193,7% so cung ky. Tren nen LNTT 457 ty cua 2025, moi 5,5 diem thue ~ 25 ty LNST moi nam. Noi vao dinh gia: mo hinh da neo 19,5% tu 2026 tro di; ai con dung 14% lich su se thoi LNST 2027F len ~8%.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>cho</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>GHI HOI TO 14/09/2026. LY DO MUA (17-19/08/2026): MSB qua bo loc MA200 + RS va giu suat cuoi bang xep hang top-40%, voi loi the co cau duoc goi ten la CASA 28,94% thuoc nhom cao nhat he thong va DANG DI LEN (26,54% -&gt; 26,42% -&gt; 28,94%), keo theo NIM 3,22% cao hon binh quan nganh 2,87% khoang 35 diem co ban, va CIR cai thien deu 41,39% (2022) -&gt; 36,14% (2025). Do la luan diem 'ngan hang co nen tien gui re va bo may dang re di'. Phieu 14/09 KHONG bac luan diem nay — cac su kien van dung — nhung do duoc rang loi the do CHUA BAO VE DUOC BIEN: CASA phuc hoi trong 2025 ma NIM van roi 3,57% -&gt; 3,22% trong dung nam do.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>Chờ thẩm định</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Khac</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>STB</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>loai</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>ro co ban chua chot</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>loai</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>cho</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>PHU QUYET BUOC 3 — phieu tham dinh 13/09/2026, het han 12/12/2026. Nam cong phu quyet DEU KHONG bat; phieu chet o DIEM: truc A 0 + truc B 1 + truc C 0 = 1/6, vua duoi tran 2 vua co truc bang 0 (thoa ca hai dieu kien phu quyet). TRUC A = 0: ROE 2025 10,34% va TTM den 30/06/2026 ~5,2% deu duoi COE 15,38% — hai trong ba ky do gan nhat duoi chi phi von. Nam duy nhat vuot la 2024 (20,03%) va no vuot nho chi phi tin dung 0,39% tren du no binh quan (so 1,95% cua 2025), dung nam ma NHNN ket luan trich lap du phong chua dung quy dinh — diem quan sat duy nhat chong lai muc 0 lai la diem quan sat da bi co quan quan ly dat dau hoi. TRUC C = 0: QD 1869 (cong bo 16-17/08/2025, phat 975 trieu, 6 vi pham, 28 kien nghi) ket luan PHAN LOAI TAI SAN CO va TRICH LAP DU PHONG chua dung quy dinh — ben co toan bo ho so tin dung noi rang so lieu dau vao sai, la dang bang chung nguoc nang nhat co the co cho mot truc cham chat luong cong bo. Cong them 3.789 ty 'dich vu khac' (21,7% tong thu nhap hoat dong 6T/2026, +2.408 ty YoY) khong co thuyet minh. TRUC B = 1: nen tien gui ban le 647.939 ty voi LDR 98,2% la loi the cau truc that, nhung CHUA quy doi duoc thanh bien co loi — CASA 18,9% (2022) -&gt; 16,5%, chi phi von tren tai san sinh loi 3,81% (2024) -&gt; 4,42%, NIM 2,81% da THAP HON binh quan nganh 2,87%, nhan su 18.659 -&gt; 13.078. Thay doi cau truc nganh bat loi nhung do duoc nen khong roi xuong 0. DO BEN KET LUAN: doc rong tay nhat cho truc A (chi lay 3 nam tai chinh 2023-2025, vut bo ky soat xet moi nhat) van ra 2/6 = VAN PHU QUYET. Phai dong thoi bo qua ky soat xet moi nhat VA ket luan thanh tra VA cham truc B muc 2 (du CASA/NIM deu di xuong) moi ra duoc 'Dat'.</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>Bán</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Chờ thẩm định</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Khac</t>
         </is>
@@ -3710,7 +3710,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MSB</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -3730,22 +3730,22 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>dat</t>
+          <t>loai</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>cho</t>
+          <t>chua</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>GHI HOI TO 14/09/2026. LY DO MUA (17-19/08/2026): MSB qua bo loc MA200 + RS va giu suat cuoi bang xep hang top-40%, voi loi the co cau duoc goi ten la CASA 28,94% thuoc nhom cao nhat he thong va DANG DI LEN (26,54% -&gt; 26,42% -&gt; 28,94%), keo theo NIM 3,22% cao hon binh quan nganh 2,87% khoang 35 diem co ban, va CIR cai thien deu 41,39% (2022) -&gt; 36,14% (2025). Do la luan diem 'ngan hang co nen tien gui re va bo may dang re di'. Phieu 14/09 KHONG bac luan diem nay — cac su kien van dung — nhung do duoc rang loi the do CHUA BAO VE DUOC BIEN: CASA phuc hoi trong 2025 ma NIM van roi 3,57% -&gt; 3,22% trong dung nam do.</t>
+          <t>Loai khoi danh muc do van de co ban (nguoi tham dinh phu quyet o buoc 3, ngay 01/09/2026). Phu quyet dinh tinh thang moi tin hieu ky thuat, ke ca 7/7 checklist ngay 25/08.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -3772,7 +3772,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>DHC</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -3797,13 +3797,17 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>chua</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>BA LUAN DIEM — phieu 13/09/2026, nhip C. Chi viet duoc vi nhip B DAT; day la ma DUY NHAT trong bon phieu di het quy trinh. (1) CU SOC PHONG KHE LA CU SOC CUNG VA DA CHUYEN THANH BIEN LOI NHUAN, khong dung o tin tuc: ~200 co so dong cua tu dau 2025 rut ~2 trieu tan/nam = 22-26% nang luc nganh, thieu hut 601.000 tan trong 7 thang dau 2026. Gia ban giay cua DHC di tu ~9.002 d/kg (Q2/2025) len 10.442 d/kg (Q2/2026), +16%. Co che: DHC song bang CHENH LECH gia, gia OCC ton kho dung o 4.800 d/kg trong khi gia ban tang 1.440 d/kg, nen gan nhu toan bo muc tang roi thang xuong bien — bien gop 11,8% (2024) -&gt; 24,2% (6T/2026). Noi vao dinh gia: bien gop 23,5% cua 2026F la GIA DINH TRUNG TAM cua toan bo mo hinh. (2) DHC CHUYEN LOI NHUAN THANH TIEN TOT HON MOI MA TRONG NHOM SO SANH, VA DIEU DO DA DUOC KIEM O DAY CHU KY CHU KHONG PHAI O DINH: dong tien HD cong don 2023-2025 = 144,2% LNST cong don; nam te nhat 2024 khi bien gop roi xuong 11,8% dong tien van 656,2 ty = 2,7 lan LNST 242,2 ty; no rong AM 339 ty tai 30/06/2026. Co che: vong quay ngan vi mua va ban deu giao ngay, khau hao 111,1 ty/nam chay tren day chuyen DA TRA XONG, va khong mot dong phai thu ben lien quan nao phai cho thu. Noi vao dinh gia: day la thu cho phep tai tro 1.814 ty con lai cua Giao Long 3 MA KHONG CAN TANG VON — tuc khong pha loang nguoi dang cam co phieu. (3) UU DAI THUE HET HAN LA BUOC NHAY CHI PHI VINH VIEN phai neo vao MOI nam du phong, khong phai bien dong mot lan: uu dai giam 50% cua Giao Long giai doan 2 het hieu luc 31/12/2025; thue suat hieu dung di tu 14,0% (2025) len 19,5% (6T/2026), chi phi thue hien hanh +193,7% so cung ky. Tren nen LNTT 457 ty cua 2025, moi 5,5 diem thue ~ 25 ty LNST moi nam. Noi vao dinh gia: mo hinh da neo 19,5% tu 2026 tro di; ai con dung 14% lich su se thoi LNST 2027F len ~8%.</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -3892,7 +3896,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>HCM</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -3912,7 +3916,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>loai</t>
+          <t>dat</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -3920,11 +3924,7 @@
           <t>chua</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Loai khoi danh muc do van de co ban (nguoi tham dinh phu quyet o buoc 3, ngay 01/09/2026). Phu quyet dinh tinh thang moi tin hieu ky thuat, ke ca 7/7 checklist ngay 25/08.</t>
-        </is>
-      </c>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -4068,224 +4068,224 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>LPB</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>loai</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>ro co ban chua chot</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>cho</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>Bán</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Khac</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>DGW</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>dat</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>ro co ban chua chot</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>chua</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>chua</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>Chờ thẩm định</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Khac</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>LPB</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>loai</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>Chờ thẩm định</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Khac</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>BSR</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>ro co ban chua chot</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>dat</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>cho</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>Bán</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Khac</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Khac</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>PHP</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>dat</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>ro co ban chua chot</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>chua</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>chua</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>Chờ thẩm định</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Khac</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>BSR</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>dat</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>ro co ban chua chot</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>dat</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>dat</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K25" s="7" t="inlineStr">
-        <is>
-          <t>Bán</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>Chờ thẩm định</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Khac</t>
         </is>
@@ -4456,7 +4456,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>SSB</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -4510,7 +4510,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SSB</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">

</xml_diff>